<commit_message>
feat: orquestrador gerar.py + primeira página gerada (site/index.html, estado.json)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -20581,7 +20581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="D5:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="8.7109375" customWidth="1" style="31" min="1" max="3"/>
@@ -20599,10 +20599,6 @@
     <col width="8.7109375" customWidth="1" style="31" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5">
       <c r="D5" s="30" t="inlineStr">
         <is>
@@ -20724,10 +20720,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1">
       <c r="D11" s="32" t="inlineStr">
         <is>
@@ -20747,7 +20739,7 @@
         </is>
       </c>
       <c r="E12" s="30">
-        <f>SUM(Mané!K5:K76)</f>
+        <f>SUM('Mané'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20758,7 +20750,7 @@
         </is>
       </c>
       <c r="E13" s="30">
-        <f>SUM(AH!K5:K76)</f>
+        <f>SUM('AH'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20769,7 +20761,7 @@
         </is>
       </c>
       <c r="E14" s="30">
-        <f>SUM(Romanelli!K5:K76)</f>
+        <f>SUM('Romanelli'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20780,7 +20772,7 @@
         </is>
       </c>
       <c r="E15" s="30">
-        <f>SUM(Su!K5:K76)</f>
+        <f>SUM('Su'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20791,7 +20783,7 @@
         </is>
       </c>
       <c r="E16" s="30">
-        <f>SUM(Rodrigo!K5:K76)</f>
+        <f>SUM('Rodrigo'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20802,7 +20794,7 @@
         </is>
       </c>
       <c r="E17" s="30">
-        <f>SUM(Beda!K5:K76)</f>
+        <f>SUM('Beda'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20813,7 +20805,7 @@
         </is>
       </c>
       <c r="E18" s="30">
-        <f>SUM(Mauro!K5:K76)</f>
+        <f>SUM('Mauro'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20824,7 +20816,7 @@
         </is>
       </c>
       <c r="E19" s="30">
-        <f>SUM(Pedro!K5:K76)</f>
+        <f>SUM('Pedro'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20835,7 +20827,7 @@
         </is>
       </c>
       <c r="E20" s="30">
-        <f>SUM(Caio!K5:K76)+10</f>
+        <f>SUM('Caio'!K5:K76)+10</f>
         <v/>
       </c>
     </row>
@@ -20846,7 +20838,7 @@
         </is>
       </c>
       <c r="E21" s="30">
-        <f>SUM(Biral!K5:K76)</f>
+        <f>SUM('Biral'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20857,7 +20849,7 @@
         </is>
       </c>
       <c r="E22" s="30">
-        <f>SUM(Paulo!K5:K76)</f>
+        <f>SUM('Paulo'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20879,7 +20871,7 @@
         </is>
       </c>
       <c r="E24" s="30">
-        <f>SUM(Kim!K5:K76)+10</f>
+        <f>SUM('Kim'!K5:K76)+10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: atualização manual 26/06 — jogos 55-60 (Mané 119)
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -3445,13 +3445,17 @@
           <t>Equador</t>
         </is>
       </c>
-      <c r="D59" s="13" t="n"/>
+      <c r="D59" s="13" t="n">
+        <v>2</v>
+      </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n"/>
+      <c r="F59" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="G59" s="12" t="inlineStr">
         <is>
           <t>Alemanha</t>
@@ -3482,13 +3486,17 @@
           <t>Curaçau</t>
         </is>
       </c>
-      <c r="D60" s="13" t="n"/>
+      <c r="D60" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n"/>
+      <c r="F60" s="13" t="n">
+        <v>2</v>
+      </c>
       <c r="G60" s="12" t="inlineStr">
         <is>
           <t>Costa do Marfim</t>
@@ -3519,13 +3527,17 @@
           <t>Turquia</t>
         </is>
       </c>
-      <c r="D61" s="13" t="n"/>
+      <c r="D61" s="13" t="n">
+        <v>3</v>
+      </c>
       <c r="E61" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F61" s="13" t="n"/>
+      <c r="F61" s="13" t="n">
+        <v>2</v>
+      </c>
       <c r="G61" s="12" t="inlineStr">
         <is>
           <t>EUA</t>
@@ -3556,13 +3568,17 @@
           <t>Paraguai</t>
         </is>
       </c>
-      <c r="D62" s="13" t="n"/>
+      <c r="D62" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="E62" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F62" s="13" t="n"/>
+      <c r="F62" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
           <t>Austrália</t>
@@ -3593,13 +3609,17 @@
           <t>Tunísia</t>
         </is>
       </c>
-      <c r="D63" s="13" t="n"/>
+      <c r="D63" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="E63" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F63" s="13" t="n"/>
+      <c r="F63" s="13" t="n">
+        <v>3</v>
+      </c>
       <c r="G63" s="12" t="inlineStr">
         <is>
           <t>Holanda</t>
@@ -3630,13 +3650,17 @@
           <t>Japão</t>
         </is>
       </c>
-      <c r="D64" s="13" t="n"/>
+      <c r="D64" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F64" s="13" t="n"/>
+      <c r="F64" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
           <t>Suécia</t>
@@ -20768,11 +20792,11 @@
     <row r="15">
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>Su</t>
+          <t>Beda</t>
         </is>
       </c>
       <c r="E15" s="30">
-        <f>SUM('Su'!K5:K76)</f>
+        <f>SUM('Beda'!K5:K76)</f>
         <v/>
       </c>
     </row>
@@ -20790,55 +20814,55 @@
     <row r="17">
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>Beda</t>
+          <t>Su</t>
         </is>
       </c>
       <c r="E17" s="30">
-        <f>SUM('Beda'!K5:K76)</f>
+        <f>SUM('Su'!K5:K76)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="D18" s="30" t="inlineStr">
         <is>
-          <t>Mauro</t>
+          <t>Pedro</t>
         </is>
       </c>
       <c r="E18" s="30">
-        <f>SUM('Mauro'!K5:K76)</f>
+        <f>SUM('Pedro'!K5:K76)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>Pedro</t>
+          <t>Mauro</t>
         </is>
       </c>
       <c r="E19" s="30">
-        <f>SUM('Pedro'!K5:K76)</f>
+        <f>SUM('Mauro'!K5:K76)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>Caio</t>
+          <t>Biral</t>
         </is>
       </c>
       <c r="E20" s="30">
-        <f>SUM('Caio'!K5:K76)+10</f>
+        <f>SUM('Biral'!K5:K76)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>Biral</t>
+          <t>Caio</t>
         </is>
       </c>
       <c r="E21" s="30">
-        <f>SUM('Biral'!K5:K76)</f>
+        <f>SUM('Caio'!K5:K76)+10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: setas de variação persistem entre runs (baseline = última ordem estável, não o run anterior)
O robô roda várias vezes/dia; a lógica antiga comparava com o estado do run
anterior e sobrescrevia a baseline, então runs sem jogos novos zeravam tudo
pra '–'. Agora a baseline só avança quando a classificação muda — extraído em
calcular_variacao() (pura, com testes em tests/test_variacao.py). estado.json
ganha campo ordem_anterior; semeado com a ordem de 25/06 p/ mostrar o movimento da noite.
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>

</xml_diff>

<commit_message>
feat(mata-mata): merge dos palpites da 1a rodada (R32) — 11 de 13
Jogos 73-88 preenchidos nas abas de Beda, Biral, Caio, Kim, Mané,
Mauro, Paulo, Pedro, Rodrigo, Romanelli e Su (16 jogos cada).
AH e Camps ainda sem palpite (não enviaram até o prazo das 16h);
abas em branco = zero na rodada por enquanto.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -4793,22 +4793,6 @@
         </is>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -4830,7 +4814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -8041,10 +8025,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -8084,10 +8074,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>4</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -8127,10 +8123,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -8170,10 +8172,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -8213,10 +8221,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -8256,10 +8270,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -8299,10 +8319,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -8342,10 +8368,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -8385,10 +8417,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -8428,10 +8466,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -8471,10 +8515,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -8514,10 +8564,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>3</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -8557,10 +8613,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>2</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -8600,10 +8662,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -8643,10 +8711,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>3</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -8686,10 +8760,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -8715,22 +8795,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -8750,7 +8814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -12727,22 +12791,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -12762,7 +12810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -16121,10 +16169,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -16164,10 +16218,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -16207,10 +16267,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -16250,10 +16316,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -16293,10 +16365,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -16336,10 +16414,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>2</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>3</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -16379,10 +16463,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -16422,10 +16512,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>2</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -16465,10 +16561,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -16508,10 +16610,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -16551,10 +16659,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -16594,10 +16708,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -16637,10 +16757,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>2</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -16680,10 +16806,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -16723,10 +16855,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>3</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -16766,10 +16904,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>2</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -16795,22 +16939,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -16832,7 +16960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -20860,22 +20988,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -20897,7 +21009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" thickBot="1">
@@ -24104,10 +24216,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -24147,10 +24265,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>3</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -24190,10 +24314,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -24233,10 +24363,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>2</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -24276,10 +24412,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -24319,10 +24461,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -24362,10 +24510,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -24405,10 +24559,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>1</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>2</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -24448,10 +24608,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -24491,10 +24657,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -24534,10 +24706,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -24577,10 +24755,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>3</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -24620,10 +24804,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>3</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -24663,10 +24853,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>3</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -24706,10 +24902,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>2</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -24749,10 +24951,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -24778,22 +24986,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -25370,7 +25562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -28624,10 +28816,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -28667,10 +28865,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -28710,10 +28914,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -28753,10 +28963,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -28796,10 +29012,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -28839,10 +29061,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -28882,10 +29110,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -28925,10 +29159,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -28968,10 +29208,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -29011,10 +29257,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -29054,10 +29306,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -29097,10 +29355,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -29140,10 +29404,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -29183,10 +29453,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>3</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -29226,10 +29502,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -29269,10 +29551,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -29298,22 +29586,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -29335,7 +29607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -32698,10 +32970,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>21</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -32741,10 +33019,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>3</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -32784,10 +33068,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -32827,10 +33117,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -32870,10 +33166,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -32913,10 +33215,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -32956,10 +33264,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -32999,10 +33313,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -33042,10 +33362,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -33085,10 +33411,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -33128,10 +33460,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -33171,10 +33509,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -33214,10 +33558,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -33257,10 +33607,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>3</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -33300,10 +33656,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -33343,10 +33705,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -33372,22 +33740,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -33409,7 +33761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -36768,10 +37120,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -36811,10 +37169,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -36854,10 +37218,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>3</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -36897,10 +37267,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -36940,10 +37316,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>4</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -36983,10 +37365,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>3</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -37026,10 +37414,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -37069,10 +37463,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -37112,10 +37512,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>4</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -37155,10 +37561,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -37198,10 +37610,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -37241,10 +37659,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -37284,10 +37708,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>3</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -37327,10 +37757,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -37370,10 +37806,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>3</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -37413,10 +37855,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -37442,22 +37890,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -37479,7 +37911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -40832,10 +41264,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -40875,10 +41313,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -40918,10 +41362,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -40961,10 +41411,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -41004,10 +41460,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -41047,10 +41509,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -41090,10 +41558,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -41133,10 +41607,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>2</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -41176,10 +41656,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -41219,10 +41705,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -41262,10 +41754,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -41305,10 +41803,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -41348,10 +41852,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -41391,10 +41901,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>3</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -41434,10 +41950,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -41477,10 +41999,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -41506,22 +42034,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -41543,7 +42055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -44806,10 +45318,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -44849,10 +45367,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>2</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -44892,10 +45416,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>3</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -44935,10 +45465,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -44978,10 +45514,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -45021,10 +45563,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -45064,10 +45612,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -45107,10 +45661,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -45150,10 +45710,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -45193,10 +45759,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>3</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -45236,10 +45808,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -45279,10 +45857,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -45322,10 +45906,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -45365,10 +45955,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -45408,10 +46004,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -45451,10 +46053,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -45480,22 +46088,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -45517,7 +46109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -48788,10 +49380,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -48831,10 +49429,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>3</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -48874,10 +49478,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>3</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -48917,10 +49527,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>2</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -48960,10 +49576,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>4</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -49003,10 +49625,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -49046,10 +49674,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>3</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -49089,10 +49723,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -49132,10 +49772,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -49175,10 +49821,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>3</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -49218,10 +49870,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -49261,10 +49919,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>3</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -49304,10 +49968,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -49347,10 +50017,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -49390,10 +50066,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>3</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -49433,10 +50115,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -49462,22 +50150,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -49499,7 +50171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -52778,10 +53450,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -52821,10 +53499,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -52864,10 +53548,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -52907,10 +53597,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -52950,10 +53646,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -52993,10 +53695,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -53036,10 +53744,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -53079,10 +53793,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>2</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -53122,10 +53842,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -53165,10 +53891,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -53208,10 +53940,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -53251,10 +53989,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -53294,10 +54038,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -53337,10 +54087,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>2</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -53380,10 +54136,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -53423,10 +54185,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>2</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -53452,22 +54220,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -53489,7 +54241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -56832,10 +57584,16 @@
           <t>África do Sul</t>
         </is>
       </c>
+      <c r="D77" t="n">
+        <v>2</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -56875,10 +57633,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -56918,10 +57682,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>3</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -56961,10 +57731,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>2</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -57004,10 +57780,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -57047,10 +57829,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -57090,10 +57878,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -57133,10 +57927,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>2</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -57176,10 +57976,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -57219,10 +58025,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -57262,10 +58074,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -57305,10 +58123,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -57348,10 +58172,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -57391,10 +58221,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -57434,10 +58270,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -57477,10 +58319,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -57506,22 +58354,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
feat(mata-mata): merge atrasado do AH (André) — jogos 74-88, jogo 73 zerado
Exceção da regra confirmada pelo Caio: quem não enviou no prazo perde só o
1º jogo (73, África do Sul × Canadá), não a rodada toda. André enviou atrasado;
gravados os jogos 74-88 na aba dele, jogo 73 deixado em branco (= 0).
Camps ainda não enviou (segue zerado). Mesma regra valerá pra ele.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -4799,22 +4799,6 @@
         </is>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -4836,7 +4820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -8817,22 +8801,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -8852,7 +8820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -12829,22 +12797,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -12864,7 +12816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -16993,22 +16945,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -17030,7 +16966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -20427,10 +20363,16 @@
           <t>Alemanha</t>
         </is>
       </c>
+      <c r="D78" t="n">
+        <v>3</v>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -20470,10 +20412,16 @@
           <t>Holanda</t>
         </is>
       </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F79" t="n">
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -20513,10 +20461,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D80" t="n">
+        <v>2</v>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -20556,10 +20510,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -20599,10 +20559,16 @@
           <t>Costa do Marfim</t>
         </is>
       </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -20642,10 +20608,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -20685,10 +20657,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -20728,10 +20706,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -20771,10 +20755,16 @@
           <t>Bélgica</t>
         </is>
       </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -20814,10 +20804,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -20857,10 +20853,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D88" t="n">
+        <v>3</v>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -20900,10 +20902,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -20943,10 +20951,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D90" t="n">
+        <v>3</v>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -20986,10 +21000,16 @@
           <t>Colômbia</t>
         </is>
       </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -21029,10 +21049,16 @@
           <t>Austrália</t>
         </is>
       </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -21058,22 +21084,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -21095,7 +21105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" thickBot="1">
@@ -25072,22 +25082,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -25664,7 +25658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -29688,22 +29682,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -29725,7 +29703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -33858,22 +33836,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -33895,7 +33857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -38024,22 +37986,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -38061,7 +38007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -42184,22 +42130,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -42221,7 +42151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -46254,22 +46184,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -46291,7 +46205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -50332,22 +50246,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -50369,7 +50267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -54418,22 +54316,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -54455,7 +54337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -58568,22 +58450,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
feat(mata-mata): Excel bate com o site nos jogos de pênaltis + aba Regras
A fórmula K do Excel só conhece o sinal V/E/D, então divergia do site num
jogo de pênaltis (ex.: quem apostou a vitória do time que passou marcava no
site mas não na K — Kim, jogo 75). Agora gerar.py grava a K desses jogos com
o valor exato do motor (nova fixar_pontos_penaltis em planilha.py) — célula e
somas do Excel passam a bater com o site. Também atualizei a aba Regras com a
regra de pênaltis/empate (decisão de 01/07/2026).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -4835,22 +4835,6 @@
         </is>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -4872,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -8853,22 +8837,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -8888,7 +8856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -12865,22 +12833,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -12900,7 +12852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -17029,22 +16981,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -17066,7 +17002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -21184,22 +21120,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -21221,7 +21141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" thickBot="1">
@@ -25198,22 +25118,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -25544,7 +25448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -25777,6 +25681,76 @@
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="27" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- Mata-mata (fase eliminatoria) - penaltis e empates:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Vale o placar ate o fim da prorrogacao (120 min). Os penaltis NAO contam como gols.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Os 2 pontos do resultado (Regra A) vao para quem ACERTOU o empate dos 120 min OU para quem apontou o time que se CLASSIFICOU nos penaltis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Assim, apostar empate pode valer os 5 pontos (Regras A+B+C), igual a fase de grupos - desde que crave o placar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Exemplo: jogo 1x1 nos 120 min, classifica o time B nos penaltis:</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Aposta 1x1 = 5 pontos (cravou o empate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Aposta 2x2 = 2 pontos (acertou que ia empatar, errou o placar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Aposta vitoria do time B (ex.: 0x1) = 2 pontos (apontou quem passou).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Aposta vitoria do time A = 0 no resultado (Regras B e C ainda valem pelo placar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>(Atualizacao de 01/07/2026: antes, apostar empate no mata-mata nao marcava os 2 pontos do resultado; agora marca.)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25790,7 +25764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -29814,22 +29788,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -29851,7 +29809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -33984,22 +33942,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -34021,7 +33963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -38150,22 +38092,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -38187,7 +38113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -42310,22 +42236,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -42347,7 +42257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -46380,22 +46290,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -46417,7 +46311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -50458,22 +50352,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -50495,7 +50373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -54544,22 +54422,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -54581,7 +54443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -58694,22 +58556,6 @@
         <v/>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
Merge palpites das oitavas (89-96): recupera pontuação perdida no fim de semana
A bateria do PC morreu sábado antes de eu commitar o merge, então o robô
pontuou os jogos 89-92 com as abas de palpites vazias (todos zerados nas
oitavas). Re-apliquei o merge das 12 planilhas (todas entregues antes do 1º
jogo) sobre a mestre já com os resultados do fim de semana e rodei gerar.py.

Oitavas jogadas: J89 França, J90 Marrocos, J91 Noruega (Brasil eliminado),
J92 Inglaterra. Classificação corrigida (líder Beda 197). Camps fora = 0.
J93-96 pontuam sozinhos quando saírem os placares (palpites já gravados).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -9246,10 +9246,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -9289,10 +9295,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -9332,10 +9344,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>3</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -9375,10 +9393,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -9418,10 +9442,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -9461,10 +9491,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -9504,10 +9540,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -9547,10 +9589,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -18088,10 +18136,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -18131,10 +18185,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>3</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -18174,10 +18234,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>3</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -18217,10 +18283,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -18260,10 +18332,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -18303,10 +18381,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>2</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -18346,10 +18430,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -18389,10 +18479,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -22576,10 +22672,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -22619,10 +22721,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>3</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -22662,10 +22770,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>3</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -22705,10 +22819,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>0</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -22748,10 +22868,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>2</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -22791,10 +22917,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -22834,10 +22966,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -22877,10 +23015,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -26923,10 +27067,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>8</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -26966,10 +27116,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>4</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -27009,10 +27165,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>4</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -27052,10 +27214,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>2</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -27095,10 +27263,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>2</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -27138,10 +27312,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>3</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -27181,10 +27361,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -27500,33 +27686,33 @@
     <row r="18">
       <c r="D18" s="30" t="inlineStr">
         <is>
-          <t>Paulo</t>
+          <t>Pedro</t>
         </is>
       </c>
       <c r="E18" s="30">
-        <f>SUM('Paulo'!K5:K108)</f>
+        <f>SUM('Pedro'!K5:K108)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>Pedro</t>
+          <t>Caio</t>
         </is>
       </c>
       <c r="E19" s="30">
-        <f>SUM('Pedro'!K5:K108)</f>
+        <f>SUM('Caio'!K5:K108)+10</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>Caio</t>
+          <t>Paulo</t>
         </is>
       </c>
       <c r="E20" s="30">
-        <f>SUM('Caio'!K5:K108)+10</f>
+        <f>SUM('Paulo'!K5:K108)</f>
         <v/>
       </c>
     </row>
@@ -31942,10 +32128,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -31985,10 +32177,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -32028,10 +32226,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -32071,10 +32275,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -32114,10 +32324,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -32157,10 +32373,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>2</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -32200,10 +32422,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>2</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -32243,10 +32471,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -36445,10 +36679,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -36488,10 +36728,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -36531,10 +36777,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -36574,10 +36826,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -36617,10 +36875,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -36660,10 +36924,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -36703,10 +36973,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -36746,10 +37022,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -40944,10 +41226,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>4</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -40987,10 +41275,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -41030,10 +41324,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -41073,10 +41373,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>2</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -41116,10 +41422,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -41159,10 +41471,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>3</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -41202,10 +41520,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -41245,10 +41569,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -45437,10 +45767,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -45480,10 +45816,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -45523,10 +45865,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -45566,10 +45914,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -45609,10 +45963,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -45652,10 +46012,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -45695,10 +46061,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>2</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -45738,10 +46110,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -49840,10 +50218,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -49883,10 +50267,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -49926,10 +50316,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>3</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -49969,10 +50365,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>2</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -50012,10 +50414,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>2</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -50055,10 +50463,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -50098,10 +50512,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -50141,10 +50561,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -54251,10 +54677,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -54294,10 +54726,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>3</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -54337,10 +54775,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -54380,10 +54824,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -54423,10 +54873,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>2</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -54466,10 +54922,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -54509,10 +54971,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -54552,10 +55020,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -58670,10 +59144,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -58713,10 +59193,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -58756,10 +59242,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -58799,10 +59291,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -58842,10 +59340,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -58885,10 +59389,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -58928,10 +59438,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -58971,10 +59487,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -63153,10 +63675,16 @@
           <t>Paraguai</t>
         </is>
       </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -63196,10 +63724,16 @@
           <t>Canadá</t>
         </is>
       </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -63239,10 +63773,16 @@
           <t>Brasil</t>
         </is>
       </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -63282,10 +63822,16 @@
           <t>México</t>
         </is>
       </c>
+      <c r="D96" t="n">
+        <v>2</v>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -63325,10 +63871,16 @@
           <t>Portugal</t>
         </is>
       </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -63368,10 +63920,16 @@
           <t>EUA</t>
         </is>
       </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -63411,10 +63969,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D99" t="n">
+        <v>2</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -63454,10 +64018,16 @@
           <t>Suíça</t>
         </is>
       </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Estende mestre com as QUARTAS (jogos 97-100)
Oitavas fechadas (J93 Espanha, J94 Bélgica, J95 Argentina, J96 Suíça nos
pênaltis). `python -m scripts.preencher_vencedores` derivou os confrontos da
mestre e gerou o molde + adicionou os jogos 97-100 (Resultados + 13 abas, com a
fórmula K; placares/palpites em branco). Quartas:
  J97 França×Marrocos · J98 Espanha×Bélgica · J99 Noruega×Inglaterra · J100 Argentina×Suíça
Classificação intacta (jogos novos somam 0 até ter placar+palpite). Molde
gitignored (só local, pra circular no grupo). Merge dos palpites após o prazo
(1º jogo J97, 09/07 17h BRT).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -5249,14 +5249,162 @@
         </is>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -5278,7 +5426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -9647,14 +9795,178 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -9674,7 +9986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -13991,14 +14303,178 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -14018,7 +14494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -18535,14 +19011,178 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -18564,7 +19204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -23070,14 +23710,178 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -23099,7 +23903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" thickBot="1">
@@ -27458,14 +28262,178 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -27485,7 +28453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D5:P24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="8.7109375" customWidth="1" style="31" min="1" max="3"/>
@@ -27503,6 +28471,10 @@
     <col width="8.7109375" customWidth="1" style="31" min="17" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="D5" s="30" t="inlineStr">
         <is>
@@ -27624,6 +28596,10 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1">
       <c r="D11" s="32" t="inlineStr">
         <is>
@@ -28112,7 +29088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -32524,14 +33500,178 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -32553,7 +33693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -37074,14 +38214,178 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -37103,7 +38407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -41620,14 +42924,178 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -41649,7 +43117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -46160,14 +47628,178 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -46189,7 +47821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -50610,14 +52242,178 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -50639,7 +52435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -55068,14 +56864,178 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -55097,7 +57057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -59534,14 +61494,178 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -59563,7 +61687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -64064,14 +66188,178 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Marrocos</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="I101">
+        <f>H101</f>
+        <v/>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="K101">
+        <f>IF(AND(ISNUMBER(D101),ISNUMBER(F101),ISNUMBER(Resultados!D101),ISNUMBER(Resultados!F101)),IF(SIGN(D101-F101)=SIGN(Resultados!D101-Resultados!F101),2,0)+IF(D101=Resultados!D101,1,0)+IF(F101=Resultados!F101,1,0)+IF(D101+F101=Resultados!D101+Resultados!F101,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Bélgica</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I102">
+        <f>H102</f>
+        <v/>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="K102">
+        <f>IF(AND(ISNUMBER(D102),ISNUMBER(F102),ISNUMBER(Resultados!D102),ISNUMBER(Resultados!F102)),IF(SIGN(D102-F102)=SIGN(Resultados!D102-Resultados!F102),2,0)+IF(D102=Resultados!D102,1,0)+IF(F102=Resultados!F102,1,0)+IF(D102+F102=Resultados!D102+Resultados!F102,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Noruega</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I103">
+        <f>H103</f>
+        <v/>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K103">
+        <f>IF(AND(ISNUMBER(D103),ISNUMBER(F103),ISNUMBER(Resultados!D103),ISNUMBER(Resultados!F103)),IF(SIGN(D103-F103)=SIGN(Resultados!D103-Resultados!F103),2,0)+IF(D103=Resultados!D103,1,0)+IF(F103=Resultados!F103,1,0)+IF(D103+F103=Resultados!D103+Resultados!F103,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Suíça</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="I104">
+        <f>H104</f>
+        <v/>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="K104">
+        <f>IF(AND(ISNUMBER(D104),ISNUMBER(F104),ISNUMBER(Resultados!D104),ISNUMBER(Resultados!F104)),IF(SIGN(D104-F104)=SIGN(Resultados!D104-Resultados!F104),2,0)+IF(D104=Resultados!D104,1,0)+IF(F104=Resultados!F104,1,0)+IF(D104+F104=Resultados!D104+Resultados!F104,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
Merge palpites das QUARTAS (10 enviaram; faltam Mané e Kim; Camps fora do mata-mata)
Grava J97-100 das 10 planilhas recebidas na pasta "planilha respostas quartas".
Regera site/estado (0 jogos novos — quartas ainda não jogadas).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -9813,10 +9813,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -9856,10 +9862,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -9899,10 +9911,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -9942,10 +9960,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -19037,10 +19061,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>3</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -19080,10 +19110,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -19123,10 +19159,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -19166,10 +19208,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -23740,10 +23788,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -23783,10 +23837,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>3</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -23826,10 +23886,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -23869,10 +23935,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -33530,10 +33602,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -33573,10 +33651,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -33616,10 +33700,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -33659,10 +33749,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -38248,10 +38344,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -38291,10 +38393,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -38334,10 +38442,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -38377,10 +38491,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -42962,10 +43082,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -43005,10 +43131,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -43048,10 +43180,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>2</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -43091,10 +43229,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -47670,10 +47814,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -47713,10 +47863,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -47756,10 +47912,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -47799,10 +47961,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -52288,10 +52456,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -52331,10 +52505,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -52374,10 +52554,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -52417,10 +52603,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>2</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -56914,10 +57106,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -56957,10 +57155,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -57000,10 +57204,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -57043,10 +57253,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>3</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -61548,10 +61764,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -61591,10 +61813,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -61634,10 +61862,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -61677,10 +61911,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Merge palpite do Mané nas QUARTAS (11 enviaram; falta só Kim; Camps fora)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -66486,10 +66486,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -66529,10 +66535,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -66572,10 +66584,16 @@
           <t>Noruega</t>
         </is>
       </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -66615,10 +66633,16 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SEMIS: mestre estendida com J101-102 (Franca x Espanha, Inglaterra x Argentina)
Todas as quartas decididas (J97 Franca 2x0 Marrocos, J98 Espanha 2x1
Belgica, J99 Noruega 1x2 Inglaterra, J100 Argentina 3x1 Suica). Rodei
preencher_vencedores -> molde gerado (local/gitignored, pronto pro grupo)
+ mestre estendida com jogos 101-102 (pontos zerados = classificacao
intacta; robo pontua sozinho quando as semis sairem).

Chaveamento: M101 Franca x Espanha (14/07 16h BRT = PRAZO, Dallas),
M102 Inglaterra x Argentina (15/07 16h, Atlanta).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -5429,10 +5429,84 @@
         </is>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -5454,7 +5528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -10019,10 +10093,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -10042,7 +10198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -14531,10 +14687,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -14554,7 +14792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -19267,10 +19505,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -19292,7 +19612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -23994,10 +24314,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -24019,7 +24421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" thickBot="1">
@@ -28550,10 +28952,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -28573,7 +29057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D5:P24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="8.7109375" customWidth="1" style="31" min="1" max="3"/>
@@ -28591,6 +29075,10 @@
     <col width="8.7109375" customWidth="1" style="31" min="17" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="D5" s="30" t="inlineStr">
         <is>
@@ -28712,6 +29200,10 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1">
       <c r="D11" s="32" t="inlineStr">
         <is>
@@ -29200,7 +29692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -33808,10 +34300,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -33833,7 +34407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -38550,10 +39124,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -38575,7 +39231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -43288,10 +43944,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -43313,7 +44051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -48020,10 +48758,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -48045,7 +48865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -52662,10 +53482,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -52687,7 +53589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -57312,10 +58214,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -57337,7 +58321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.28515625" customWidth="1" min="10" max="10"/>
@@ -61970,10 +62954,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -61995,7 +63061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="9.5703125" customWidth="1" min="1" max="1"/>
@@ -66692,10 +67758,92 @@
         <v/>
       </c>
     </row>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="I105">
+        <f>H105</f>
+        <v/>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K105">
+        <f>IF(AND(ISNUMBER(D105),ISNUMBER(F105),ISNUMBER(Resultados!D105),ISNUMBER(Resultados!F105)),IF(SIGN(D105-F105)=SIGN(Resultados!D105-Resultados!F105),2,0)+IF(D105=Resultados!D105,1,0)+IF(F105=Resultados!F105,1,0)+IF(D105+F105=Resultados!D105+Resultados!F105,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I106">
+        <f>H106</f>
+        <v/>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K106">
+        <f>IF(AND(ISNUMBER(D106),ISNUMBER(F106),ISNUMBER(Resultados!D106),ISNUMBER(Resultados!F106)),IF(SIGN(D106-F106)=SIGN(Resultados!D106-Resultados!F106),2,0)+IF(D106=Resultados!D106,1,0)+IF(F106=Resultados!F106,1,0)+IF(D106+F106=Resultados!D106+Resultados!F106,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
SEMIS: merge dos palpites (10 de 12) — J101-102
10 participantes entregaram (AH, Beda, Biral, Caio, Mané, Mauro,
Pedro, Rodrigo, Romanelli, Su); faltaram Paulo e Kim (Camps fora do
mata-mata). Semis ainda sem placar — palpites gravados; robô pontua
sozinho quando J101/J102 saírem.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -10109,10 +10109,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -10152,10 +10158,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -19525,10 +19537,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -19568,10 +19586,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -24336,10 +24360,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -24379,10 +24409,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -34318,10 +34354,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -34361,10 +34403,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -39144,10 +39192,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -39187,10 +39241,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -43966,10 +44026,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -44009,10 +44075,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>3</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -48782,10 +48854,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -48825,10 +48903,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -58242,10 +58326,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -58285,10 +58375,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -62984,10 +63080,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -63027,10 +63129,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -67790,10 +67898,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -67833,10 +67947,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SEMIS: Paulo entrou no merge (11 de 12) — J101-102
Paulo mandou (Caio tinha esquecido de pôr o arquivo na pasta).
Re-merge idempotente: agora 11 participantes com os 2 jogos; falta só
o Kim (Camps fora do mata-mata). Semis ainda sem placar.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -53592,10 +53592,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -53635,10 +53641,16 @@
           <t>Inglaterra</t>
         </is>
       </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: preparar última rodada (3º lugar + Final, jogos 103-104)
3º lugar J103 = perdedores das semis (França x Inglaterra);
Final J104 = vencedores (Espanha x Argentina). Molde de 2 jogos gerado
(local/gitignored) e mestre estendida com 103-104 (zerados = classificação
intacta). Scripts reconfigurados p/ a rodada final:
- preencher_vencedores: novo perdedor() + FINAL_BRACKET (V/P por feeder)
- preparar_rodada: PRIMEIRO_JOGO=103, título/confrontos da rodada
- merge_respostas: pasta "planilha respostas final", PRIMEIRO_JOGO=103
- .gitignore + LEIA-ME da pasta nova

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -5519,8 +5519,84 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -10205,8 +10281,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -14801,8 +14961,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -19633,8 +19877,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -24456,8 +24784,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -29096,8 +29508,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F1:I1"/>
@@ -29117,7 +29613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D5:P24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col width="8.7109375" customWidth="1" style="31" min="1" max="3"/>
@@ -29135,6 +29631,10 @@
     <col width="8.7109375" customWidth="1" style="31" min="17" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="D5" s="30" t="inlineStr">
         <is>
@@ -29256,6 +29756,10 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1">
       <c r="D11" s="32" t="inlineStr">
         <is>
@@ -34450,8 +34954,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -39288,8 +39876,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -44122,8 +44794,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -48950,8 +49706,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -53688,8 +54528,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -58434,8 +59358,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -63188,8 +64196,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>
@@ -68006,8 +69098,92 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3º Lugar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>França</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I107">
+        <f>H107</f>
+        <v/>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="K107">
+        <f>IF(AND(ISNUMBER(D107),ISNUMBER(F107),ISNUMBER(Resultados!D107),ISNUMBER(Resultados!F107)),IF(SIGN(D107-F107)=SIGN(Resultados!D107-Resultados!F107),2,0)+IF(D107=Resultados!D107,1,0)+IF(F107=Resultados!F107,1,0)+IF(D107+F107=Resultados!D107+Resultados!F107,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espanha</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I108">
+        <f>H108</f>
+        <v/>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="K108">
+        <f>IF(AND(ISNUMBER(D108),ISNUMBER(F108),ISNUMBER(Resultados!D108),ISNUMBER(Resultados!F108)),IF(SIGN(D108-F108)=SIGN(Resultados!D108-Resultados!F108),2,0)+IF(D108=Resultados!D108,1,0)+IF(F108=Resultados!F108,1,0)+IF(D108+F108=Resultados!D108+Resultados!F108,1,0),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="F1:I1"/>

</xml_diff>

<commit_message>
feat: merge da última rodada (3º lugar + Final) — Copa encerrada
Resultados: J103 França 4x6 Inglaterra (3º = Inglaterra), J104 Espanha 1x0
Argentina (Espanha CAMPEÃ). Merge de 10 palpites (Su só a final; Paulo/Kim
não enviaram -> zeram a rodada pela regra; Camps fora). Repontuado via gerar.py,
site == estado.json (13/13).

Pódio final: 1º Beda 225 (R$325), 2º Rodrigo 217 (R$195), 3º AH 212 (R$130).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABELA_APOSTAS_-_COPA_2026.xlsx
+++ b/TABELA_APOSTAS_-_COPA_2026.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Beda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Su" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Biral" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mané" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Caio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Camps " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AH" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Kim" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Regras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedro" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mauro" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rodrigo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paulo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Su" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biral" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mané" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camps " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Romanelli" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AH" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kim" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pontos" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="alex">#REF!</definedName>
@@ -10307,10 +10307,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -10350,10 +10356,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>3</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -19903,10 +19915,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>3</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -19946,10 +19964,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>3</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -24810,10 +24834,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -24853,10 +24883,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -29823,22 +29859,22 @@
     <row r="16">
       <c r="D16" s="30" t="inlineStr">
         <is>
-          <t>Caio</t>
+          <t>Su</t>
         </is>
       </c>
       <c r="E16" s="30">
-        <f>SUM('Caio'!K5:K108)+10</f>
+        <f>SUM('Su'!K5:K108)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>Su</t>
+          <t>Caio</t>
         </is>
       </c>
       <c r="E17" s="30">
-        <f>SUM('Su'!K5:K108)</f>
+        <f>SUM('Caio'!K5:K108)+10</f>
         <v/>
       </c>
     </row>
@@ -29867,33 +29903,33 @@
     <row r="20">
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>Paulo</t>
+          <t>Mauro</t>
         </is>
       </c>
       <c r="E20" s="30">
-        <f>SUM('Paulo'!K5:K108)</f>
+        <f>SUM('Mauro'!K5:K108)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>Mauro</t>
+          <t>Biral</t>
         </is>
       </c>
       <c r="E21" s="30">
-        <f>SUM('Mauro'!K5:K108)</f>
+        <f>SUM('Biral'!K5:K108)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="30" t="inlineStr">
         <is>
-          <t>Biral</t>
+          <t>Paulo</t>
         </is>
       </c>
       <c r="E22" s="30">
-        <f>SUM('Biral'!K5:K108)</f>
+        <f>SUM('Paulo'!K5:K108)</f>
         <v/>
       </c>
     </row>
@@ -34972,10 +35008,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -35015,10 +35057,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -39894,10 +39942,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -39937,10 +39991,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -44812,10 +44872,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>3</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -44855,10 +44921,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -49724,10 +49796,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -49767,10 +49845,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -59419,10 +59503,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -64214,10 +64304,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>3</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -64257,10 +64353,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -69116,10 +69218,16 @@
           <t>França</t>
         </is>
       </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -69159,10 +69267,16 @@
           <t>Espanha</t>
         </is>
       </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>

</xml_diff>